<commit_message>
Extended Excom appointment letters template added
</commit_message>
<xml_diff>
--- a/team-emails/sampledata.xlsx
+++ b/team-emails/sampledata.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ABC\Documents\acm-automation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ABC\Documents\acm-automation\team-emails\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A75792A-3C53-4F8E-8A6D-F1629DD6A1D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93A82316-9141-4627-97BF-5B13DEFBD1FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{7D79C001-8A5B-4E0F-BFF1-DA2C69A5F7B5}"/>
   </bookViews>
@@ -47,19 +47,19 @@
     <t>position</t>
   </si>
   <si>
-    <t xml:space="preserve">Musab Ali </t>
+    <t>email</t>
+  </si>
+  <si>
+    <t>mmak.lughat@gmail.com</t>
+  </si>
+  <si>
+    <t>Musab</t>
   </si>
   <si>
     <t>Co Head</t>
   </si>
   <si>
-    <t>Automation</t>
-  </si>
-  <si>
-    <t>email</t>
-  </si>
-  <si>
-    <t>mmak.lughat@gmail.com</t>
+    <t>Automations</t>
   </si>
 </sst>
 </file>
@@ -446,11 +446,13 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="21.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -464,21 +466,21 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" t="s">
         <v>7</v>
-      </c>
-      <c r="B2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D2" t="s">
-        <v>5</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" xr:uid="{6C973147-62CA-4DF5-A911-B46CBA687BD7}"/>
+    <hyperlink ref="A2" r:id="rId1" xr:uid="{5B31AF6E-4FA3-4297-9D3A-D825F1165920}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>